<commit_message>
Created master validation module
Built validators for duplicate ids, missing values, data types and business rules
</commit_message>
<xml_diff>
--- a/data/raw/sales.xlsx
+++ b/data/raw/sales.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Goku eta vaina e seria\Portafolio\Python - Excel to PostgreSQL Pipeline\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4E5CCF9A-E1BA-49B9-A4A5-438380B51B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFA2D344-76A3-4C44-8CE2-6E7A80E2C722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{51FF519F-AC21-4AB1-BA5A-06C40468EE10}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" xr2:uid="{51FF519F-AC21-4AB1-BA5A-06C40468EE10}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -65,9 +65,6 @@
     <t>region</t>
   </si>
   <si>
-    <t>Alice Smith</t>
-  </si>
-  <si>
     <t>Laptop</t>
   </si>
   <si>
@@ -108,6 +105,9 @@
   </si>
   <si>
     <t>Desk</t>
+  </si>
+  <si>
+    <t>Alice Kingsleigh</t>
   </si>
 </sst>
 </file>
@@ -143,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -157,10 +157,7 @@
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -504,32 +501,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>10001</v>
       </c>
@@ -537,13 +534,13 @@
         <v>46204</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>9</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>10</v>
       </c>
       <c r="F2" s="1">
         <v>1</v>
@@ -552,7 +549,7 @@
         <v>899.99</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -563,13 +560,13 @@
         <v>46204</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>13</v>
-      </c>
       <c r="E3" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F3" s="1">
         <v>2</v>
@@ -578,7 +575,7 @@
         <v>19.989999999999998</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -589,13 +586,13 @@
         <v>46205</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>17</v>
       </c>
       <c r="F4" s="1">
         <v>1</v>
@@ -604,7 +601,7 @@
         <v>149.5</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -615,13 +612,13 @@
         <v>46206</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>19</v>
-      </c>
       <c r="E5" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F5" s="1">
         <v>1</v>
@@ -630,7 +627,7 @@
         <v>59.99</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -641,13 +638,13 @@
         <v>46207</v>
       </c>
       <c r="C6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>22</v>
-      </c>
       <c r="E6" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F6" s="1">
         <v>1</v>
@@ -656,7 +653,7 @@
         <v>299.99</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>